<commit_message>
parties sync, order placement etc
</commit_message>
<xml_diff>
--- a/phase0/SalesOn-WooCommerce-Product-Mapping-Review.xlsx
+++ b/phase0/SalesOn-WooCommerce-Product-Mapping-Review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\codes\mycoolstar\phase0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C80B67-E2C3-45F2-ABB1-06AE1678E630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35ED6921-B73F-4DF0-A0C2-E0D62EC20C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3941" uniqueCount="2240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3947" uniqueCount="2245">
   <si>
     <t>SalesOn - WooCommerce Product Mapping Review</t>
   </si>
@@ -6759,6 +6759,21 @@
   </si>
   <si>
     <t>shipping</t>
+  </si>
+  <si>
+    <t>Warehouse</t>
+  </si>
+  <si>
+    <t>HB Akeda</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>MCS</t>
+  </si>
+  <si>
+    <t>Website ID</t>
   </si>
 </sst>
 </file>
@@ -7152,19 +7167,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="75" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="4" max="4" width="19.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -7172,28 +7188,40 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>903</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D5" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E5" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>352</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>2242</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -7201,7 +7229,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -7209,7 +7237,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -7217,7 +7245,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -7225,12 +7253,12 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -7238,7 +7266,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -7246,7 +7274,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -10477,7 +10505,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I125"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -10488,9 +10516,11 @@
     <col min="6" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="11" max="11" width="16.81640625" customWidth="1"/>
+    <col min="12" max="12" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>35</v>
       </c>
@@ -10518,8 +10548,14 @@
       <c r="I1" s="4" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="K1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -10548,7 +10584,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -10577,7 +10613,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -10606,7 +10642,7 @@
         <v>19.096</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -10635,7 +10671,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -10661,7 +10697,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -10687,7 +10723,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -10716,7 +10752,7 @@
         <v>46.872</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -10745,7 +10781,7 @@
         <v>33.851999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -10774,7 +10810,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -10803,7 +10839,7 @@
         <v>53.816000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -10832,7 +10868,7 @@
         <v>39.06</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -10861,7 +10897,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -10890,7 +10926,7 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -10913,7 +10949,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -15629,7 +15665,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -15640,7 +15676,7 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
@@ -15660,7 +15696,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -15679,8 +15715,11 @@
       <c r="F2" t="s">
         <v>546</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2">
+        <v>130418</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -15700,7 +15739,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -15720,7 +15759,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -15740,7 +15779,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -15760,7 +15799,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -15780,7 +15819,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -15800,7 +15839,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -15820,7 +15859,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -15837,7 +15876,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -15854,7 +15893,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -15874,7 +15913,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -15894,7 +15933,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -15914,7 +15953,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -15934,7 +15973,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>